<commit_message>
automatic update 2026-10-05 12:57:32
</commit_message>
<xml_diff>
--- a/Streamlit/Data/definition.xlsx
+++ b/Streamlit/Data/definition.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4051" uniqueCount="1411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4055" uniqueCount="1415">
   <si>
     <t>Process</t>
   </si>
@@ -3234,7 +3234,7 @@
     <t>Bayesian inference is a statistical method for updating the probability of a hypothesis based on new evidence., "It works by using Bayes theorem to calculate the posterior distribution of the hypothesis given the new evidence, taking into account prior knowledge and uncertainty.", Bayesian inference is important because it allows us to quantify uncertainty and make predictions in complex systems with incomplete data., Typical applications include Bayesian regression, Bayesian classification, and Bayesian time series analysis.</t>
   </si>
   <si>
-    <t>{What the analytical method is: Expectation-Maximization (EM) is a statistical algorithm for finding maximum likelihood estimates of parameters in probabilistic models., How it works: The EM algorithm iteratively updates the model parameters and the unobserved variables until convergence, alternating between two steps: expectation (E-step) and maximization (M-step)., Why it is important: EM is essential for handling missing data and identifying underlying patterns in datasets. It is widely used in various applications, including clustering, classification, and dimensionality reduction., Its typical applications: EM is commonly employed in machine learning tasks such as cluster analysis, anomaly detection, and feature extraction.}</t>
+    <t>Expectation-Maximization (EM) is an iterative optimization algorithm for estimating parameters of probabilistic models when the data contain latent or unobserved variables, alternating between an Expectation (E) step that estimates the latent-variable distribution and a Maximization (M) step that updates model parameters. It is particularly relevant to problems such as Gaussian mixture model clustering, missing-data estimation, and other latent-variable models where direct maximum-likelihood estimation is difficult. EM is important because it transforms a difficult optimization involving hidden information into a sequence of more tractable estimation problems, with each iteration guaranteed not to decrease the observed-data likelihood under standard conditions. The general EM algorithm was formally named and popularized by Arthur Dempster, Nan Laird, and Donald Rubin in their influential 1977 paper, although related iterative estimation techniques existed earlier.</t>
   </si>
   <si>
     <t>{What the analytical method is: Decision Rules are a type of analytical technique that involves making decisions based on predefined rules., How it works: The decision-making process follows a set of rules, which are applied to input data to generate output or predictions., Why it is important: Decision Rules provide a transparent and interpretable way to make predictions or classify instances., Its typical applications: Decision Rules are often used in classification problems where the goal is to predict a categorical label based on input features.}</t>
@@ -3288,7 +3288,7 @@
     <t>{What the analytical method is: Convolutional Neural Networks (CNNs) are a type of neural network architecture., How it works: They work by applying multiple convolution and downsampling operations followed by fully connected layers to classify images., Why it is important: CNNs have been instrumental in achieving state-of-the-art results in image classification tasks, object detection, and segmentation., Its typical applications: CNNs are widely used in computer vision tasks such as image classification, object detection, and image generation.}</t>
   </si>
   <si>
-    <t>{What the analytical method is: As Features is a technique used to select relevant features from a dataset, often in the context of classification or regression problems., How it works: It typically involves evaluating the importance or relevance of each feature using various metrics such as mutual information, correlation coefficient, or recursive feature elimination (RFE), and selecting the top-ranked features for further analysis or modeling., Why it is important: Feature selection is crucial in machine learning to prevent overfitting, improve model interpretability, reduce dimensionality, and enhance prediction performance. By identifying the most relevant features, analysts can focus on the most informative variables and develop more accurate models., Its typical applications: As Features has been applied extensively in various domains such as text classification, image analysis, gene expression data analysis, and recommender systems.}</t>
+    <t>practice of transforming information, model outputs, or derived measurements into variables that serve as inputs to another statistical or machine-learning model. For example, cluster assignments, embeddings, predicted probabilities, dates, text-derived measurements, or aggregated historical behavior can all be represented as features for a downstream model. This approach is relevant to feature engineering, representation learning, ensemble methods, and multi-stage ML pipelines because it allows information discovered in one processing step to become predictive information for another. It is important because model performance often depends as much on how useful information is represented as features as on the choice of learning algorithm itself, although care must be taken to prevent problems such as target leakage.</t>
   </si>
   <si>
     <t>Translation invariance is a property of neural networks that refers to their ability to maintain performance even when the input data is shifted, rotated, or transformed in some other way., This property is achieved through the use of convolutional and pooling layers in deep learning architectures, which allow the network to learn features that are invariant to these transformations., Translation invariance is an important concept in computer vision and image processing because it enables the extraction of meaningful features from images without being sensitive to their spatial location or orientation., Typically, translation invariance is applied in tasks such as image classification, object detection, and segmentation.</t>
@@ -3408,7 +3408,7 @@
     <t>{What the analytical method is: Contrastive learning is a type of unsupervised machine learning algorithm that aims to learn representations by contrasting similar and dissimilar inputs., How it works: "The method involves two main steps: positive pair sampling, where similar input pairs are generated, and negative pair sampling, where dissimilar input pairs are generated. A contrastive loss function is then used to update the models parameters.", Why it is important: Contrastive learning has been shown to be effective in learning robust and transferable representations, which can improve the performance of downstream tasks., Its typical applications: Contrastive learning has applications in image classification, object detection, and recommendation systems.}</t>
   </si>
   <si>
-    <t>Autoencoding is a type of unsupervised learning algorithm that learns to compress and reconstruct input data., It works by defining an encoder network that maps the input data to a lower-dimensional latent space, and a decoder network that maps the latent space back to the original input data., The importance of autoencoding lies in its ability to learn compact representations of high-dimensional data, which can be useful for dimensionality reduction, anomaly detection, and generative modeling., Autoencoding is typically applied in areas such as image compression, text processing, and recommender systems.</t>
+    <t>Autoencoding is an unsupervised representation-learning technique in which a neural network learns to reconstruct its input after passing it through an intermediate latent representation, typically using an encoder and decoder. It is relevant when learning compact representations of high-dimensional data, particularly for dimensionality reduction, feature extraction, denoising, anomaly detection, and generative modeling. Autoencoding is important because the reconstruction objective allows useful features and structure to be learned from unlabeled data, while constraints such as a bottleneck, sparsity, or noise prevent the model from simply copying its input. Autoencoders developed from neural-network research into efficient data representations, with important early work appearing in the 1980s and later becoming prominent in deep learning through multilayer and variational architectures.</t>
   </si>
   <si>
     <t>Metric learning is a subfield of machine learning that focuses on learning distance metrics from data., It works by minimizing the difference between the learned metric and the true underlying metric, often using kernel-based methods or probabilistic approaches., Metric learning is important because it allows for more effective clustering, classification, and other tasks that rely on similarity measurements., It has applications in image recognition, natural language processing, and information retrieval.</t>
@@ -3512,7 +3512,7 @@
     <t>Linear Support Vector Classification (LinearSVC) is a supervised machine learning algorithm. It works by finding the optimal hyperplane that separates classes in the feature space, maximally preserving class separability. This method is important because it provides a simple and interpretable way to perform classification tasks with linear decision boundaries. Typical applications include image classification, text classification, and recommender systems.</t>
   </si>
   <si>
-    <t>MeanShift is a non-parametric, adaptive density-based clustering algorithm that automatically determines the number of clusters in the data. It works by iteratively shifting the centroids of overlapping Gaussian distributions towards higher-density regions until convergence. This method is important because it can handle complex, high-dimensional datasets and does not require any prior knowledge about the underlying structure. Typical applications include image segmentation, object tracking, and bioinformatics.</t>
+    <t>MeanShift is a non-parametric clustering algorithm that iteratively moves candidate cluster centers toward regions of higher estimated data density until they converge on local density modes. Unlike methods such as K-means, it does not require the number of clusters to be specified beforehand, but instead relies heavily on a bandwidth parameter that determines the neighborhood used for estimating density. It is relevant when clusters may have irregular distributions or when the appropriate number of clusters is unknown, although it can become computationally expensive for large or high-dimensional datasets. MeanShift originated in pattern-recognition research by Fukunaga and Hostetler in 1975 and was later popularized particularly in computer vision and image segmentation.</t>
   </si>
   <si>
     <t>NuSVR is a type of Support Vector Regression algorithm that uses a nu-regression parameter to control the fraction of training errors. It works by mapping the input data into a high-dimensional feature space using a kernel function, and then finding the optimal hyperplane in this space. The importance of NuSVR lies in its ability to handle non-linear relationships between inputs and outputs, making it useful for regression problems with complex underlying structures. Typically, NuSVR is applied to real-world problems such as forecasting, modeling, or prediction.</t>
@@ -3907,6 +3907,15 @@
   </si>
   <si>
     <t>Manifold is different than linear interpolation, manifold is a slow gradual change, linear is averaging/combining.</t>
+  </si>
+  <si>
+    <t>You do not specify the number of clusters in mean shift they are determined based on the density, it is most useful in applications of spatial hotspots, image segmentation, computer vision/object tracking, and exploratory clustering where the number of groups isn't known..</t>
+  </si>
+  <si>
+    <t>EM looks to address the circular problem; I could estimate my model parameters easily if I knew the hidden information—but I don't know the hidden information, while I could estimate the hidden information if I knew the model parameters—but I don't know those either.</t>
+  </si>
+  <si>
+    <t>An autoencoder is particularly useful when you have many features and potentially nonlinear relationships. For example, imagine 500 behavioral variables describing how a credit-union member interacts with different products and channels. Instead of feeding all 500 variables into another model, an autoencoder might learn 30 latent features representing underlying behavioral patterns. PCA is a linear representation.</t>
   </si>
   <si>
     <t>https://raw.githubusercontent.com/derek-dewald/d_functions/main/images/cosine_similiarity.png</t>
@@ -4020,6 +4029,28 @@
 $$
 y_i(\mathbf{w} \cdot \mathbf{x}_i + b) \geq 1, \quad \forall i
 $$</t>
+  </si>
+  <si>
+    <t>### Expectation-Maximization (EM) Process
+**1. Initialize Model Parameters**  
+Start with initial estimates (or guesses) for the parameters of the model.
+↓  
+**2. Expectation Step (E-Step)**  
+Using the current model parameters, estimate the **latent (unobserved) variables**.  
+For a Gaussian Mixture Model, calculate the probability that each observation belongs to each Gaussian distribution.
+↓  
+**3. Maximization Step (M-Step)**  
+Using the estimated latent-variable probabilities from the E-Step, calculate new model parameters that **maximize the likelihood of the observed data**.  
+For a Gaussian Mixture Model, update the mean, variance, and mixture weight of each Gaussian distribution.
+↓  
+**4. Repeat E-Step and M-Step**  
+Use the newly estimated model parameters to perform another E-Step, followed by another M-Step.
+↓  
+**5. Convergence**  
+Continue alternating between the E-Step and M-Step until the model parameters or likelihood change by less than a specified threshold.
+---
+**In simple terms:**
+`Initialize → Estimate Hidden Variables (E) → Update Model Parameters (M) → Repeat → Converge`</t>
   </si>
   <si>
     <t>### **Definition:**
@@ -6169,10 +6200,10 @@
         <v>745</v>
       </c>
       <c r="G96" s="1" t="s">
-        <v>1264</v>
+        <v>1267</v>
       </c>
       <c r="H96" t="s">
-        <v>1269</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="97" spans="1:7">
@@ -6189,7 +6220,7 @@
         <v>746</v>
       </c>
       <c r="G97" s="1" t="s">
-        <v>1264</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="98" spans="1:7">
@@ -6875,7 +6906,7 @@
         <v>793</v>
       </c>
       <c r="H146" t="s">
-        <v>1270</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="147" spans="1:8">
@@ -7119,7 +7150,7 @@
         <v>810</v>
       </c>
       <c r="H163" t="s">
-        <v>1271</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="164" spans="1:8">
@@ -7136,7 +7167,7 @@
         <v>811</v>
       </c>
       <c r="H164" t="s">
-        <v>1272</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="165" spans="1:8">
@@ -7153,10 +7184,10 @@
         <v>812</v>
       </c>
       <c r="F165" s="1" t="s">
-        <v>1263</v>
+        <v>1266</v>
       </c>
       <c r="H165" t="s">
-        <v>1273</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="166" spans="1:8">
@@ -7978,7 +8009,7 @@
         <v>853</v>
       </c>
       <c r="G228" s="1" t="s">
-        <v>1265</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="229" spans="1:14">
@@ -8006,7 +8037,7 @@
         <v>854</v>
       </c>
       <c r="G230" s="1" t="s">
-        <v>1266</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="231" spans="1:14">
@@ -8048,7 +8079,7 @@
         <v>856</v>
       </c>
       <c r="H233" t="s">
-        <v>1274</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="234" spans="1:14">
@@ -8065,7 +8096,7 @@
         <v>857</v>
       </c>
       <c r="H234" t="s">
-        <v>1275</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="235" spans="1:14">
@@ -8164,7 +8195,7 @@
         <v>265</v>
       </c>
       <c r="N240" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="241" spans="1:14">
@@ -8193,7 +8224,7 @@
         <v>266</v>
       </c>
       <c r="N241" t="s">
-        <v>1384</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="242" spans="1:14">
@@ -8271,10 +8302,10 @@
         <v>156</v>
       </c>
       <c r="K244" t="s">
-        <v>1282</v>
+        <v>1286</v>
       </c>
       <c r="L244" t="s">
-        <v>1297</v>
+        <v>1301</v>
       </c>
       <c r="M244" t="s">
         <v>269</v>
@@ -8332,7 +8363,7 @@
         <v>173</v>
       </c>
       <c r="L246" t="s">
-        <v>1298</v>
+        <v>1302</v>
       </c>
       <c r="M246" t="s">
         <v>271</v>
@@ -8358,16 +8389,16 @@
         <v>155</v>
       </c>
       <c r="K247" t="s">
-        <v>1283</v>
+        <v>1287</v>
       </c>
       <c r="L247" t="s">
-        <v>1299</v>
+        <v>1303</v>
       </c>
       <c r="M247" t="s">
         <v>272</v>
       </c>
       <c r="N247" t="s">
-        <v>1385</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="248" spans="1:14">
@@ -8419,13 +8450,13 @@
         <v>165</v>
       </c>
       <c r="L249" t="s">
-        <v>1297</v>
+        <v>1301</v>
       </c>
       <c r="M249" t="s">
         <v>274</v>
       </c>
       <c r="N249" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="250" spans="1:14">
@@ -8448,13 +8479,13 @@
         <v>170</v>
       </c>
       <c r="L250" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M250" t="s">
         <v>275</v>
       </c>
       <c r="N250" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="251" spans="1:14">
@@ -8483,7 +8514,7 @@
         <v>276</v>
       </c>
       <c r="N251" t="s">
-        <v>1387</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="252" spans="1:14">
@@ -8541,7 +8572,7 @@
         <v>278</v>
       </c>
       <c r="N253" t="s">
-        <v>1385</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="254" spans="1:14">
@@ -8570,7 +8601,7 @@
         <v>279</v>
       </c>
       <c r="N254" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="255" spans="1:14">
@@ -8599,7 +8630,7 @@
         <v>280</v>
       </c>
       <c r="N255" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="256" spans="1:14">
@@ -8651,13 +8682,13 @@
         <v>170</v>
       </c>
       <c r="L257" t="s">
-        <v>1301</v>
+        <v>1305</v>
       </c>
       <c r="M257" t="s">
         <v>282</v>
       </c>
       <c r="N257" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="258" spans="1:14">
@@ -8709,7 +8740,7 @@
         <v>167</v>
       </c>
       <c r="L259" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M259" t="s">
         <v>284</v>
@@ -8744,7 +8775,7 @@
         <v>285</v>
       </c>
       <c r="N260" t="s">
-        <v>1390</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="261" spans="1:14">
@@ -8773,7 +8804,7 @@
         <v>286</v>
       </c>
       <c r="N261" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="262" spans="1:14">
@@ -8802,7 +8833,7 @@
         <v>287</v>
       </c>
       <c r="N262" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="263" spans="1:14">
@@ -8825,13 +8856,13 @@
         <v>167</v>
       </c>
       <c r="L263" t="s">
-        <v>1302</v>
+        <v>1306</v>
       </c>
       <c r="M263" t="s">
         <v>288</v>
       </c>
       <c r="N263" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="264" spans="1:14">
@@ -8854,7 +8885,7 @@
         <v>170</v>
       </c>
       <c r="L264" t="s">
-        <v>1303</v>
+        <v>1307</v>
       </c>
       <c r="M264" t="s">
         <v>289</v>
@@ -8883,7 +8914,7 @@
         <v>170</v>
       </c>
       <c r="L265" t="s">
-        <v>1304</v>
+        <v>1308</v>
       </c>
       <c r="M265" t="s">
         <v>290</v>
@@ -8912,7 +8943,7 @@
         <v>170</v>
       </c>
       <c r="L266" t="s">
-        <v>1305</v>
+        <v>1309</v>
       </c>
       <c r="M266" t="s">
         <v>291</v>
@@ -8941,7 +8972,7 @@
         <v>171</v>
       </c>
       <c r="L267" t="s">
-        <v>1305</v>
+        <v>1309</v>
       </c>
       <c r="M267" t="s">
         <v>292</v>
@@ -8970,13 +9001,13 @@
         <v>171</v>
       </c>
       <c r="L268" t="s">
-        <v>1306</v>
+        <v>1310</v>
       </c>
       <c r="M268" t="s">
         <v>293</v>
       </c>
       <c r="N268" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="269" spans="1:14">
@@ -9005,7 +9036,7 @@
         <v>294</v>
       </c>
       <c r="N269" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="270" spans="1:14">
@@ -9034,7 +9065,7 @@
         <v>295</v>
       </c>
       <c r="N270" t="s">
-        <v>1391</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="271" spans="1:14">
@@ -9057,13 +9088,13 @@
         <v>167</v>
       </c>
       <c r="L271" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M271" t="s">
         <v>296</v>
       </c>
       <c r="N271" t="s">
-        <v>1392</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="272" spans="1:14">
@@ -9086,13 +9117,13 @@
         <v>166</v>
       </c>
       <c r="L272" t="s">
-        <v>1307</v>
+        <v>1311</v>
       </c>
       <c r="M272" t="s">
         <v>297</v>
       </c>
       <c r="N272" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="273" spans="1:14">
@@ -9115,7 +9146,7 @@
         <v>165</v>
       </c>
       <c r="L273" t="s">
-        <v>1308</v>
+        <v>1312</v>
       </c>
       <c r="M273" t="s">
         <v>298</v>
@@ -9144,7 +9175,7 @@
         <v>167</v>
       </c>
       <c r="L274" t="s">
-        <v>1309</v>
+        <v>1313</v>
       </c>
       <c r="M274" t="s">
         <v>299</v>
@@ -9173,7 +9204,7 @@
         <v>170</v>
       </c>
       <c r="L275" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M275" t="s">
         <v>300</v>
@@ -9202,13 +9233,13 @@
         <v>167</v>
       </c>
       <c r="L276" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M276" t="s">
         <v>301</v>
       </c>
       <c r="N276" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="277" spans="1:14">
@@ -9237,7 +9268,7 @@
         <v>302</v>
       </c>
       <c r="N277" t="s">
-        <v>1385</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="278" spans="1:14">
@@ -9260,13 +9291,13 @@
         <v>167</v>
       </c>
       <c r="L278" t="s">
-        <v>1310</v>
+        <v>1314</v>
       </c>
       <c r="M278" t="s">
         <v>303</v>
       </c>
       <c r="N278" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="279" spans="1:14">
@@ -9289,13 +9320,13 @@
         <v>171</v>
       </c>
       <c r="L279" t="s">
-        <v>1311</v>
+        <v>1315</v>
       </c>
       <c r="M279" t="s">
         <v>304</v>
       </c>
       <c r="N279" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="280" spans="1:14">
@@ -9318,13 +9349,13 @@
         <v>171</v>
       </c>
       <c r="L280" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M280" t="s">
         <v>305</v>
       </c>
       <c r="N280" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="281" spans="1:14">
@@ -9347,13 +9378,13 @@
         <v>170</v>
       </c>
       <c r="L281" t="s">
-        <v>1312</v>
+        <v>1316</v>
       </c>
       <c r="M281" t="s">
         <v>306</v>
       </c>
       <c r="N281" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="282" spans="1:14">
@@ -9376,13 +9407,13 @@
         <v>165</v>
       </c>
       <c r="L282" t="s">
-        <v>1310</v>
+        <v>1314</v>
       </c>
       <c r="M282" t="s">
         <v>307</v>
       </c>
       <c r="N282" t="s">
-        <v>1391</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="283" spans="1:14">
@@ -9405,7 +9436,7 @@
         <v>167</v>
       </c>
       <c r="L283" t="s">
-        <v>1313</v>
+        <v>1317</v>
       </c>
       <c r="M283" t="s">
         <v>308</v>
@@ -9440,7 +9471,7 @@
         <v>309</v>
       </c>
       <c r="N284" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="285" spans="1:14">
@@ -9463,7 +9494,7 @@
         <v>170</v>
       </c>
       <c r="L285" t="s">
-        <v>1314</v>
+        <v>1318</v>
       </c>
       <c r="M285" t="s">
         <v>310</v>
@@ -9492,13 +9523,13 @@
         <v>167</v>
       </c>
       <c r="L286" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M286" t="s">
         <v>311</v>
       </c>
       <c r="N286" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="287" spans="1:14">
@@ -9521,13 +9552,13 @@
         <v>170</v>
       </c>
       <c r="L287" t="s">
-        <v>1305</v>
+        <v>1309</v>
       </c>
       <c r="M287" t="s">
         <v>312</v>
       </c>
       <c r="N287" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="288" spans="1:14">
@@ -9550,13 +9581,13 @@
         <v>169</v>
       </c>
       <c r="L288" t="s">
-        <v>1307</v>
+        <v>1311</v>
       </c>
       <c r="M288" t="s">
         <v>313</v>
       </c>
       <c r="N288" t="s">
-        <v>1385</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="289" spans="1:14">
@@ -9585,7 +9616,7 @@
         <v>314</v>
       </c>
       <c r="N289" t="s">
-        <v>1393</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="290" spans="1:14">
@@ -9608,7 +9639,7 @@
         <v>167</v>
       </c>
       <c r="L290" t="s">
-        <v>1315</v>
+        <v>1319</v>
       </c>
       <c r="M290" t="s">
         <v>315</v>
@@ -9637,13 +9668,13 @@
         <v>167</v>
       </c>
       <c r="L291" t="s">
-        <v>1316</v>
+        <v>1320</v>
       </c>
       <c r="M291" t="s">
         <v>316</v>
       </c>
       <c r="N291" t="s">
-        <v>1394</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="292" spans="1:14">
@@ -9663,7 +9694,7 @@
         <v>156</v>
       </c>
       <c r="K292" t="s">
-        <v>1284</v>
+        <v>1288</v>
       </c>
       <c r="L292" t="s">
         <v>222</v>
@@ -9672,7 +9703,7 @@
         <v>317</v>
       </c>
       <c r="N292" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="293" spans="1:14">
@@ -9724,7 +9755,7 @@
         <v>167</v>
       </c>
       <c r="L294" t="s">
-        <v>1317</v>
+        <v>1321</v>
       </c>
       <c r="M294" t="s">
         <v>319</v>
@@ -9753,13 +9784,13 @@
         <v>167</v>
       </c>
       <c r="L295" t="s">
-        <v>1318</v>
+        <v>1322</v>
       </c>
       <c r="M295" t="s">
         <v>320</v>
       </c>
       <c r="N295" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="296" spans="1:14">
@@ -9840,7 +9871,7 @@
         <v>170</v>
       </c>
       <c r="L298" t="s">
-        <v>1319</v>
+        <v>1323</v>
       </c>
       <c r="M298" t="s">
         <v>323</v>
@@ -9869,13 +9900,13 @@
         <v>167</v>
       </c>
       <c r="L299" t="s">
-        <v>1318</v>
+        <v>1322</v>
       </c>
       <c r="M299" t="s">
         <v>324</v>
       </c>
       <c r="N299" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="300" spans="1:14">
@@ -9898,7 +9929,7 @@
         <v>164</v>
       </c>
       <c r="L300" t="s">
-        <v>1320</v>
+        <v>1324</v>
       </c>
       <c r="M300" t="s">
         <v>325</v>
@@ -9927,13 +9958,13 @@
         <v>165</v>
       </c>
       <c r="L301" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M301" t="s">
         <v>326</v>
       </c>
       <c r="N301" t="s">
-        <v>1391</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="302" spans="1:14">
@@ -9956,7 +9987,7 @@
         <v>170</v>
       </c>
       <c r="L302" t="s">
-        <v>1311</v>
+        <v>1315</v>
       </c>
       <c r="M302" t="s">
         <v>327</v>
@@ -9985,13 +10016,13 @@
         <v>164</v>
       </c>
       <c r="L303" t="s">
-        <v>1321</v>
+        <v>1325</v>
       </c>
       <c r="M303" t="s">
         <v>328</v>
       </c>
       <c r="N303" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="304" spans="1:14">
@@ -10049,7 +10080,7 @@
         <v>330</v>
       </c>
       <c r="N305" t="s">
-        <v>1387</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="306" spans="1:14">
@@ -10072,7 +10103,7 @@
         <v>170</v>
       </c>
       <c r="L306" t="s">
-        <v>1322</v>
+        <v>1326</v>
       </c>
       <c r="M306" t="s">
         <v>331</v>
@@ -10136,7 +10167,7 @@
         <v>333</v>
       </c>
       <c r="N308" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="309" spans="1:14">
@@ -10165,7 +10196,7 @@
         <v>334</v>
       </c>
       <c r="N309" t="s">
-        <v>1391</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="310" spans="1:14">
@@ -10188,7 +10219,7 @@
         <v>167</v>
       </c>
       <c r="L310" t="s">
-        <v>1323</v>
+        <v>1327</v>
       </c>
       <c r="M310" t="s">
         <v>335</v>
@@ -10217,7 +10248,7 @@
         <v>167</v>
       </c>
       <c r="L311" t="s">
-        <v>1318</v>
+        <v>1322</v>
       </c>
       <c r="M311" t="s">
         <v>336</v>
@@ -10252,7 +10283,7 @@
         <v>337</v>
       </c>
       <c r="N312" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="313" spans="1:14">
@@ -10275,7 +10306,7 @@
         <v>165</v>
       </c>
       <c r="L313" t="s">
-        <v>1324</v>
+        <v>1328</v>
       </c>
       <c r="M313" t="s">
         <v>338</v>
@@ -10304,13 +10335,13 @@
         <v>67</v>
       </c>
       <c r="L314" t="s">
-        <v>1325</v>
+        <v>1329</v>
       </c>
       <c r="M314" t="s">
         <v>339</v>
       </c>
       <c r="N314" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="315" spans="1:14">
@@ -10397,7 +10428,7 @@
         <v>342</v>
       </c>
       <c r="N317" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="318" spans="1:14">
@@ -10426,7 +10457,7 @@
         <v>343</v>
       </c>
       <c r="N318" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="319" spans="1:14">
@@ -10478,7 +10509,7 @@
         <v>165</v>
       </c>
       <c r="L320" t="s">
-        <v>1326</v>
+        <v>1330</v>
       </c>
       <c r="M320" t="s">
         <v>345</v>
@@ -10507,13 +10538,13 @@
         <v>165</v>
       </c>
       <c r="L321" t="s">
-        <v>1327</v>
+        <v>1331</v>
       </c>
       <c r="M321" t="s">
         <v>346</v>
       </c>
       <c r="N321" t="s">
-        <v>1387</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="322" spans="1:14">
@@ -10530,19 +10561,19 @@
         <v>945</v>
       </c>
       <c r="J322" t="s">
-        <v>1281</v>
+        <v>1285</v>
       </c>
       <c r="K322" t="s">
-        <v>1285</v>
+        <v>1289</v>
       </c>
       <c r="L322" t="s">
-        <v>1328</v>
+        <v>1332</v>
       </c>
       <c r="M322" t="s">
         <v>347</v>
       </c>
       <c r="N322" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="323" spans="1:14">
@@ -10565,13 +10596,13 @@
         <v>170</v>
       </c>
       <c r="L323" t="s">
-        <v>1303</v>
+        <v>1307</v>
       </c>
       <c r="M323" t="s">
         <v>348</v>
       </c>
       <c r="N323" t="s">
-        <v>1393</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="324" spans="1:14">
@@ -10594,7 +10625,7 @@
         <v>167</v>
       </c>
       <c r="L324" t="s">
-        <v>1318</v>
+        <v>1322</v>
       </c>
       <c r="M324" t="s">
         <v>349</v>
@@ -10623,13 +10654,13 @@
         <v>170</v>
       </c>
       <c r="L325" t="s">
-        <v>1329</v>
+        <v>1333</v>
       </c>
       <c r="M325" t="s">
         <v>350</v>
       </c>
       <c r="N325" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="326" spans="1:14">
@@ -10652,13 +10683,13 @@
         <v>170</v>
       </c>
       <c r="L326" t="s">
-        <v>1330</v>
+        <v>1334</v>
       </c>
       <c r="M326" t="s">
         <v>351</v>
       </c>
       <c r="N326" t="s">
-        <v>1393</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="327" spans="1:14">
@@ -10678,7 +10709,7 @@
         <v>155</v>
       </c>
       <c r="K327" t="s">
-        <v>1286</v>
+        <v>1290</v>
       </c>
       <c r="L327" t="s">
         <v>219</v>
@@ -10687,7 +10718,7 @@
         <v>352</v>
       </c>
       <c r="N327" t="s">
-        <v>1395</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="328" spans="1:14">
@@ -10710,7 +10741,7 @@
         <v>165</v>
       </c>
       <c r="L328" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M328" t="s">
         <v>353</v>
@@ -10739,13 +10770,13 @@
         <v>167</v>
       </c>
       <c r="L329" t="s">
-        <v>1331</v>
+        <v>1335</v>
       </c>
       <c r="M329" t="s">
         <v>354</v>
       </c>
       <c r="N329" t="s">
-        <v>1392</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="330" spans="1:14">
@@ -10768,13 +10799,13 @@
         <v>165</v>
       </c>
       <c r="L330" t="s">
-        <v>1316</v>
+        <v>1320</v>
       </c>
       <c r="M330" t="s">
         <v>355</v>
       </c>
       <c r="N330" t="s">
-        <v>1392</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="331" spans="1:14">
@@ -10797,13 +10828,13 @@
         <v>167</v>
       </c>
       <c r="L331" t="s">
-        <v>1316</v>
+        <v>1320</v>
       </c>
       <c r="M331" t="s">
         <v>356</v>
       </c>
       <c r="N331" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="332" spans="1:14">
@@ -10826,7 +10857,7 @@
         <v>167</v>
       </c>
       <c r="L332" t="s">
-        <v>1302</v>
+        <v>1306</v>
       </c>
       <c r="M332" t="s">
         <v>357</v>
@@ -10852,10 +10883,10 @@
         <v>155</v>
       </c>
       <c r="K333" t="s">
-        <v>1287</v>
+        <v>1291</v>
       </c>
       <c r="L333" t="s">
-        <v>1332</v>
+        <v>1336</v>
       </c>
       <c r="M333" t="s">
         <v>358</v>
@@ -10884,13 +10915,13 @@
         <v>167</v>
       </c>
       <c r="L334" t="s">
-        <v>1326</v>
+        <v>1330</v>
       </c>
       <c r="M334" t="s">
         <v>359</v>
       </c>
       <c r="N334" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="335" spans="1:14">
@@ -10910,10 +10941,10 @@
         <v>155</v>
       </c>
       <c r="K335" t="s">
-        <v>1288</v>
+        <v>1292</v>
       </c>
       <c r="L335" t="s">
-        <v>1333</v>
+        <v>1337</v>
       </c>
       <c r="M335" t="s">
         <v>360</v>
@@ -10942,7 +10973,7 @@
         <v>167</v>
       </c>
       <c r="L336" t="s">
-        <v>1313</v>
+        <v>1317</v>
       </c>
       <c r="M336" t="s">
         <v>361</v>
@@ -10971,13 +11002,13 @@
         <v>165</v>
       </c>
       <c r="L337" t="s">
-        <v>1318</v>
+        <v>1322</v>
       </c>
       <c r="M337" t="s">
         <v>362</v>
       </c>
       <c r="N337" t="s">
-        <v>1391</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="338" spans="1:14">
@@ -11006,7 +11037,7 @@
         <v>363</v>
       </c>
       <c r="N338" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="339" spans="1:14">
@@ -11029,7 +11060,7 @@
         <v>171</v>
       </c>
       <c r="L339" t="s">
-        <v>1299</v>
+        <v>1303</v>
       </c>
       <c r="M339" t="s">
         <v>364</v>
@@ -11058,7 +11089,7 @@
         <v>171</v>
       </c>
       <c r="L340" t="s">
-        <v>1334</v>
+        <v>1338</v>
       </c>
       <c r="M340" t="s">
         <v>365</v>
@@ -11087,7 +11118,7 @@
         <v>171</v>
       </c>
       <c r="L341" t="s">
-        <v>1305</v>
+        <v>1309</v>
       </c>
       <c r="M341" t="s">
         <v>366</v>
@@ -11174,7 +11205,7 @@
         <v>167</v>
       </c>
       <c r="L344" t="s">
-        <v>1323</v>
+        <v>1327</v>
       </c>
       <c r="M344" t="s">
         <v>369</v>
@@ -11238,7 +11269,7 @@
         <v>371</v>
       </c>
       <c r="N346" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="347" spans="1:14">
@@ -11261,13 +11292,13 @@
         <v>170</v>
       </c>
       <c r="L347" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M347" t="s">
         <v>372</v>
       </c>
       <c r="N347" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="348" spans="1:14">
@@ -11290,7 +11321,7 @@
         <v>170</v>
       </c>
       <c r="L348" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M348" t="s">
         <v>373</v>
@@ -11319,13 +11350,13 @@
         <v>166</v>
       </c>
       <c r="L349" t="s">
-        <v>1335</v>
+        <v>1339</v>
       </c>
       <c r="M349" t="s">
         <v>374</v>
       </c>
       <c r="N349" t="s">
-        <v>1387</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="350" spans="1:14">
@@ -11354,7 +11385,7 @@
         <v>375</v>
       </c>
       <c r="N350" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="351" spans="1:14">
@@ -11377,13 +11408,13 @@
         <v>166</v>
       </c>
       <c r="L351" t="s">
-        <v>1335</v>
+        <v>1339</v>
       </c>
       <c r="M351" t="s">
         <v>376</v>
       </c>
       <c r="N351" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="352" spans="1:14">
@@ -11406,13 +11437,13 @@
         <v>170</v>
       </c>
       <c r="L352" t="s">
-        <v>1336</v>
+        <v>1340</v>
       </c>
       <c r="M352" t="s">
         <v>377</v>
       </c>
       <c r="N352" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="353" spans="1:14">
@@ -11435,13 +11466,13 @@
         <v>167</v>
       </c>
       <c r="L353" t="s">
-        <v>1337</v>
+        <v>1341</v>
       </c>
       <c r="M353" t="s">
         <v>378</v>
       </c>
       <c r="N353" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="354" spans="1:14">
@@ -11493,7 +11524,7 @@
         <v>170</v>
       </c>
       <c r="L355" t="s">
-        <v>1322</v>
+        <v>1326</v>
       </c>
       <c r="M355" t="s">
         <v>380</v>
@@ -11522,7 +11553,7 @@
         <v>165</v>
       </c>
       <c r="L356" t="s">
-        <v>1326</v>
+        <v>1330</v>
       </c>
       <c r="M356" t="s">
         <v>381</v>
@@ -11551,13 +11582,13 @@
         <v>167</v>
       </c>
       <c r="L357" t="s">
-        <v>1338</v>
+        <v>1342</v>
       </c>
       <c r="M357" t="s">
         <v>382</v>
       </c>
       <c r="N357" t="s">
-        <v>1392</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="358" spans="1:14">
@@ -11609,7 +11640,7 @@
         <v>167</v>
       </c>
       <c r="L359" t="s">
-        <v>1313</v>
+        <v>1317</v>
       </c>
       <c r="M359" t="s">
         <v>384</v>
@@ -11638,13 +11669,13 @@
         <v>170</v>
       </c>
       <c r="L360" t="s">
-        <v>1339</v>
+        <v>1343</v>
       </c>
       <c r="M360" t="s">
         <v>385</v>
       </c>
       <c r="N360" t="s">
-        <v>1387</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="361" spans="1:14">
@@ -11667,13 +11698,13 @@
         <v>170</v>
       </c>
       <c r="L361" t="s">
-        <v>1316</v>
+        <v>1320</v>
       </c>
       <c r="M361" t="s">
         <v>386</v>
       </c>
       <c r="N361" t="s">
-        <v>1396</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="362" spans="1:14">
@@ -11696,13 +11727,13 @@
         <v>165</v>
       </c>
       <c r="L362" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="M362" t="s">
         <v>387</v>
       </c>
       <c r="N362" t="s">
-        <v>1385</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="363" spans="1:14">
@@ -11731,7 +11762,7 @@
         <v>388</v>
       </c>
       <c r="N363" t="s">
-        <v>1397</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="364" spans="1:14">
@@ -11751,7 +11782,7 @@
         <v>155</v>
       </c>
       <c r="K364" t="s">
-        <v>1289</v>
+        <v>1293</v>
       </c>
       <c r="L364" t="s">
         <v>219</v>
@@ -11760,7 +11791,7 @@
         <v>389</v>
       </c>
       <c r="N364" t="s">
-        <v>1398</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="365" spans="1:14">
@@ -11783,13 +11814,13 @@
         <v>171</v>
       </c>
       <c r="L365" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M365" t="s">
         <v>390</v>
       </c>
       <c r="N365" t="s">
-        <v>1399</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="366" spans="1:14">
@@ -11809,16 +11840,16 @@
         <v>155</v>
       </c>
       <c r="K366" t="s">
-        <v>1286</v>
+        <v>1290</v>
       </c>
       <c r="L366" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="M366" t="s">
         <v>391</v>
       </c>
       <c r="N366" t="s">
-        <v>1385</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="367" spans="1:14">
@@ -11838,10 +11869,10 @@
         <v>155</v>
       </c>
       <c r="K367" t="s">
-        <v>1290</v>
+        <v>1294</v>
       </c>
       <c r="L367" t="s">
-        <v>1309</v>
+        <v>1313</v>
       </c>
       <c r="M367" t="s">
         <v>392</v>
@@ -11870,13 +11901,13 @@
         <v>166</v>
       </c>
       <c r="L368" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="M368" t="s">
         <v>393</v>
       </c>
       <c r="N368" t="s">
-        <v>1400</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="369" spans="1:14">
@@ -11899,13 +11930,13 @@
         <v>170</v>
       </c>
       <c r="L369" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M369" t="s">
         <v>394</v>
       </c>
       <c r="N369" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="370" spans="1:14">
@@ -11934,7 +11965,7 @@
         <v>395</v>
       </c>
       <c r="N370" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="371" spans="1:14">
@@ -11957,13 +11988,13 @@
         <v>167</v>
       </c>
       <c r="L371" t="s">
-        <v>1308</v>
+        <v>1312</v>
       </c>
       <c r="M371" t="s">
         <v>396</v>
       </c>
       <c r="N371" t="s">
-        <v>1401</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="372" spans="1:14">
@@ -11983,10 +12014,10 @@
         <v>156</v>
       </c>
       <c r="K372" t="s">
-        <v>1291</v>
+        <v>1295</v>
       </c>
       <c r="L372" t="s">
-        <v>1341</v>
+        <v>1345</v>
       </c>
       <c r="M372" t="s">
         <v>397</v>
@@ -12021,7 +12052,7 @@
         <v>398</v>
       </c>
       <c r="N373" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="374" spans="1:14">
@@ -12079,7 +12110,7 @@
         <v>400</v>
       </c>
       <c r="N375" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="376" spans="1:14">
@@ -12102,7 +12133,7 @@
         <v>166</v>
       </c>
       <c r="L376" t="s">
-        <v>1342</v>
+        <v>1346</v>
       </c>
       <c r="M376" t="s">
         <v>401</v>
@@ -12137,7 +12168,7 @@
         <v>402</v>
       </c>
       <c r="N377" t="s">
-        <v>1391</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="378" spans="1:14">
@@ -12166,7 +12197,7 @@
         <v>403</v>
       </c>
       <c r="N378" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="379" spans="1:14">
@@ -12224,7 +12255,7 @@
         <v>405</v>
       </c>
       <c r="N380" t="s">
-        <v>1391</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="381" spans="1:14">
@@ -12253,7 +12284,7 @@
         <v>406</v>
       </c>
       <c r="N381" t="s">
-        <v>1402</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="382" spans="1:14">
@@ -12282,7 +12313,7 @@
         <v>407</v>
       </c>
       <c r="N382" t="s">
-        <v>1403</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="383" spans="1:14">
@@ -12305,13 +12336,13 @@
         <v>170</v>
       </c>
       <c r="L383" t="s">
-        <v>1343</v>
+        <v>1347</v>
       </c>
       <c r="M383" t="s">
         <v>408</v>
       </c>
       <c r="N383" t="s">
-        <v>1387</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="384" spans="1:14">
@@ -12334,13 +12365,13 @@
         <v>167</v>
       </c>
       <c r="L384" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M384" t="s">
         <v>409</v>
       </c>
       <c r="N384" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="385" spans="1:14">
@@ -12363,7 +12394,7 @@
         <v>167</v>
       </c>
       <c r="L385" t="s">
-        <v>1302</v>
+        <v>1306</v>
       </c>
       <c r="M385" t="s">
         <v>410</v>
@@ -12392,13 +12423,13 @@
         <v>170</v>
       </c>
       <c r="L386" t="s">
-        <v>1344</v>
+        <v>1348</v>
       </c>
       <c r="M386" t="s">
         <v>411</v>
       </c>
       <c r="N386" t="s">
-        <v>1404</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="387" spans="1:14">
@@ -12427,7 +12458,7 @@
         <v>412</v>
       </c>
       <c r="N387" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="388" spans="1:14">
@@ -12479,7 +12510,7 @@
         <v>165</v>
       </c>
       <c r="L389" t="s">
-        <v>1337</v>
+        <v>1341</v>
       </c>
       <c r="M389" t="s">
         <v>414</v>
@@ -12502,25 +12533,25 @@
         <v>1013</v>
       </c>
       <c r="G390" s="1" t="s">
-        <v>1267</v>
+        <v>1270</v>
       </c>
       <c r="H390" t="s">
-        <v>1276</v>
+        <v>1279</v>
       </c>
       <c r="J390" t="s">
         <v>155</v>
       </c>
       <c r="K390" t="s">
-        <v>1292</v>
+        <v>1296</v>
       </c>
       <c r="L390" t="s">
-        <v>1309</v>
+        <v>1313</v>
       </c>
       <c r="M390" t="s">
         <v>415</v>
       </c>
       <c r="N390" t="s">
-        <v>1391</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="391" spans="1:14">
@@ -12549,7 +12580,7 @@
         <v>416</v>
       </c>
       <c r="N391" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="392" spans="1:14">
@@ -12572,13 +12603,13 @@
         <v>166</v>
       </c>
       <c r="L392" t="s">
-        <v>1307</v>
+        <v>1311</v>
       </c>
       <c r="M392" t="s">
         <v>417</v>
       </c>
       <c r="N392" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="393" spans="1:14">
@@ -12601,13 +12632,13 @@
         <v>166</v>
       </c>
       <c r="L393" t="s">
-        <v>1345</v>
+        <v>1349</v>
       </c>
       <c r="M393" t="s">
         <v>418</v>
       </c>
       <c r="N393" t="s">
-        <v>1384</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="394" spans="1:14">
@@ -12636,7 +12667,7 @@
         <v>419</v>
       </c>
       <c r="N394" t="s">
-        <v>1391</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="395" spans="1:14">
@@ -12688,13 +12719,13 @@
         <v>165</v>
       </c>
       <c r="L396" t="s">
-        <v>1326</v>
+        <v>1330</v>
       </c>
       <c r="M396" t="s">
         <v>421</v>
       </c>
       <c r="N396" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="397" spans="1:14">
@@ -12723,7 +12754,7 @@
         <v>422</v>
       </c>
       <c r="N397" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="398" spans="1:14">
@@ -12746,7 +12777,7 @@
         <v>173</v>
       </c>
       <c r="L398" t="s">
-        <v>1298</v>
+        <v>1302</v>
       </c>
       <c r="M398" t="s">
         <v>423</v>
@@ -12775,13 +12806,13 @@
         <v>166</v>
       </c>
       <c r="L399" t="s">
-        <v>1346</v>
+        <v>1350</v>
       </c>
       <c r="M399" t="s">
         <v>424</v>
       </c>
       <c r="N399" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="400" spans="1:14">
@@ -12810,7 +12841,7 @@
         <v>425</v>
       </c>
       <c r="N400" t="s">
-        <v>1385</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="401" spans="1:14">
@@ -12833,7 +12864,7 @@
         <v>166</v>
       </c>
       <c r="L401" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="M401" t="s">
         <v>426</v>
@@ -12862,7 +12893,7 @@
         <v>165</v>
       </c>
       <c r="L402" t="s">
-        <v>1340</v>
+        <v>1344</v>
       </c>
       <c r="M402" t="s">
         <v>427</v>
@@ -12891,13 +12922,13 @@
         <v>165</v>
       </c>
       <c r="L403" t="s">
-        <v>1334</v>
+        <v>1338</v>
       </c>
       <c r="M403" t="s">
         <v>428</v>
       </c>
       <c r="N403" t="s">
-        <v>1385</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="404" spans="1:14">
@@ -12920,7 +12951,7 @@
         <v>165</v>
       </c>
       <c r="L404" t="s">
-        <v>1347</v>
+        <v>1351</v>
       </c>
       <c r="M404" t="s">
         <v>429</v>
@@ -12978,13 +13009,13 @@
         <v>167</v>
       </c>
       <c r="L406" t="s">
-        <v>1299</v>
+        <v>1303</v>
       </c>
       <c r="M406" t="s">
         <v>431</v>
       </c>
       <c r="N406" t="s">
-        <v>1405</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="407" spans="1:14">
@@ -13004,7 +13035,7 @@
         <v>156</v>
       </c>
       <c r="K407" t="s">
-        <v>1293</v>
+        <v>1297</v>
       </c>
       <c r="L407" t="s">
         <v>239</v>
@@ -13042,7 +13073,7 @@
         <v>433</v>
       </c>
       <c r="N408" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="409" spans="1:14">
@@ -13065,13 +13096,13 @@
         <v>165</v>
       </c>
       <c r="L409" t="s">
-        <v>1302</v>
+        <v>1306</v>
       </c>
       <c r="M409" t="s">
         <v>434</v>
       </c>
       <c r="N409" t="s">
-        <v>1391</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="410" spans="1:14">
@@ -13094,13 +13125,13 @@
         <v>173</v>
       </c>
       <c r="L410" t="s">
-        <v>1348</v>
+        <v>1352</v>
       </c>
       <c r="M410" t="s">
         <v>435</v>
       </c>
       <c r="N410" t="s">
-        <v>1392</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="411" spans="1:14">
@@ -13116,6 +13147,9 @@
       <c r="D411" t="s">
         <v>1034</v>
       </c>
+      <c r="E411" t="s">
+        <v>1263</v>
+      </c>
       <c r="J411" t="s">
         <v>156</v>
       </c>
@@ -13123,13 +13157,13 @@
         <v>166</v>
       </c>
       <c r="L411" t="s">
-        <v>1349</v>
+        <v>1353</v>
       </c>
       <c r="M411" t="s">
         <v>436</v>
       </c>
       <c r="N411" t="s">
-        <v>1384</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="412" spans="1:14">
@@ -13152,13 +13186,13 @@
         <v>167</v>
       </c>
       <c r="L412" t="s">
-        <v>1350</v>
+        <v>1354</v>
       </c>
       <c r="M412" t="s">
         <v>437</v>
       </c>
       <c r="N412" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="413" spans="1:14">
@@ -13187,7 +13221,7 @@
         <v>438</v>
       </c>
       <c r="N413" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="414" spans="1:14">
@@ -13210,13 +13244,13 @@
         <v>165</v>
       </c>
       <c r="L414" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M414" t="s">
         <v>439</v>
       </c>
       <c r="N414" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="415" spans="1:14">
@@ -13239,13 +13273,13 @@
         <v>173</v>
       </c>
       <c r="L415" t="s">
-        <v>1351</v>
+        <v>1355</v>
       </c>
       <c r="M415" t="s">
         <v>440</v>
       </c>
       <c r="N415" t="s">
-        <v>1384</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="416" spans="1:14">
@@ -13268,13 +13302,13 @@
         <v>173</v>
       </c>
       <c r="L416" t="s">
-        <v>1305</v>
+        <v>1309</v>
       </c>
       <c r="M416" t="s">
         <v>441</v>
       </c>
       <c r="N416" t="s">
-        <v>1385</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="417" spans="1:14">
@@ -13297,13 +13331,13 @@
         <v>169</v>
       </c>
       <c r="L417" t="s">
-        <v>1339</v>
+        <v>1343</v>
       </c>
       <c r="M417" t="s">
         <v>442</v>
       </c>
       <c r="N417" t="s">
-        <v>1384</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="418" spans="1:14">
@@ -13326,13 +13360,13 @@
         <v>68</v>
       </c>
       <c r="L418" t="s">
-        <v>1297</v>
+        <v>1301</v>
       </c>
       <c r="M418" t="s">
         <v>443</v>
       </c>
       <c r="N418" t="s">
-        <v>1387</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="419" spans="1:14">
@@ -13348,6 +13382,12 @@
       <c r="D419" t="s">
         <v>1042</v>
       </c>
+      <c r="E419" t="s">
+        <v>1264</v>
+      </c>
+      <c r="H419" t="s">
+        <v>1280</v>
+      </c>
       <c r="J419" t="s">
         <v>156</v>
       </c>
@@ -13355,13 +13395,13 @@
         <v>166</v>
       </c>
       <c r="L419" t="s">
-        <v>1311</v>
+        <v>1315</v>
       </c>
       <c r="M419" t="s">
         <v>444</v>
       </c>
       <c r="N419" t="s">
-        <v>1406</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="420" spans="1:14">
@@ -13390,7 +13430,7 @@
         <v>445</v>
       </c>
       <c r="N420" t="s">
-        <v>1387</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="421" spans="1:14">
@@ -13413,13 +13453,13 @@
         <v>166</v>
       </c>
       <c r="L421" t="s">
-        <v>1352</v>
+        <v>1356</v>
       </c>
       <c r="M421" t="s">
         <v>446</v>
       </c>
       <c r="N421" t="s">
-        <v>1384</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="422" spans="1:14">
@@ -13442,13 +13482,13 @@
         <v>166</v>
       </c>
       <c r="L422" t="s">
-        <v>1353</v>
+        <v>1357</v>
       </c>
       <c r="M422" t="s">
         <v>447</v>
       </c>
       <c r="N422" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="423" spans="1:14">
@@ -13471,13 +13511,13 @@
         <v>446</v>
       </c>
       <c r="L423" t="s">
-        <v>1353</v>
+        <v>1357</v>
       </c>
       <c r="M423" t="s">
         <v>448</v>
       </c>
       <c r="N423" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="424" spans="1:14">
@@ -13500,13 +13540,13 @@
         <v>165</v>
       </c>
       <c r="L424" t="s">
-        <v>1333</v>
+        <v>1337</v>
       </c>
       <c r="M424" t="s">
         <v>449</v>
       </c>
       <c r="N424" t="s">
-        <v>1403</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="425" spans="1:14">
@@ -13526,16 +13566,16 @@
         <v>155</v>
       </c>
       <c r="K425" t="s">
-        <v>1294</v>
+        <v>1298</v>
       </c>
       <c r="L425" t="s">
-        <v>1333</v>
+        <v>1337</v>
       </c>
       <c r="M425" t="s">
         <v>450</v>
       </c>
       <c r="N425" t="s">
-        <v>1403</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="426" spans="1:14">
@@ -13558,13 +13598,13 @@
         <v>173</v>
       </c>
       <c r="L426" t="s">
-        <v>1354</v>
+        <v>1358</v>
       </c>
       <c r="M426" t="s">
         <v>451</v>
       </c>
       <c r="N426" t="s">
-        <v>1403</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="427" spans="1:14">
@@ -13587,7 +13627,7 @@
         <v>165</v>
       </c>
       <c r="L427" t="s">
-        <v>1355</v>
+        <v>1359</v>
       </c>
       <c r="M427" t="s">
         <v>452</v>
@@ -13616,13 +13656,13 @@
         <v>173</v>
       </c>
       <c r="L428" t="s">
-        <v>1348</v>
+        <v>1352</v>
       </c>
       <c r="M428" t="s">
         <v>453</v>
       </c>
       <c r="N428" t="s">
-        <v>1403</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="429" spans="1:14">
@@ -13645,7 +13685,7 @@
         <v>167</v>
       </c>
       <c r="L429" t="s">
-        <v>1298</v>
+        <v>1302</v>
       </c>
       <c r="M429" t="s">
         <v>454</v>
@@ -13703,7 +13743,7 @@
         <v>165</v>
       </c>
       <c r="L431" t="s">
-        <v>1356</v>
+        <v>1360</v>
       </c>
       <c r="M431" t="s">
         <v>456</v>
@@ -13738,7 +13778,7 @@
         <v>457</v>
       </c>
       <c r="N432" t="s">
-        <v>1407</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="433" spans="1:14">
@@ -13790,13 +13830,13 @@
         <v>165</v>
       </c>
       <c r="L434" t="s">
-        <v>1357</v>
+        <v>1361</v>
       </c>
       <c r="M434" t="s">
         <v>459</v>
       </c>
       <c r="N434" t="s">
-        <v>1408</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="435" spans="1:14">
@@ -13877,7 +13917,7 @@
         <v>171</v>
       </c>
       <c r="L437" t="s">
-        <v>1303</v>
+        <v>1307</v>
       </c>
       <c r="M437" t="s">
         <v>462</v>
@@ -13906,13 +13946,13 @@
         <v>173</v>
       </c>
       <c r="L438" t="s">
-        <v>1299</v>
+        <v>1303</v>
       </c>
       <c r="M438" t="s">
         <v>463</v>
       </c>
       <c r="N438" t="s">
-        <v>1390</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="439" spans="1:14">
@@ -13935,13 +13975,13 @@
         <v>170</v>
       </c>
       <c r="L439" t="s">
-        <v>1358</v>
+        <v>1362</v>
       </c>
       <c r="M439" t="s">
         <v>464</v>
       </c>
       <c r="N439" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="440" spans="1:14">
@@ -13964,13 +14004,13 @@
         <v>165</v>
       </c>
       <c r="L440" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M440" t="s">
         <v>465</v>
       </c>
       <c r="N440" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="441" spans="1:14">
@@ -14022,13 +14062,13 @@
         <v>173</v>
       </c>
       <c r="L442" t="s">
-        <v>1335</v>
+        <v>1339</v>
       </c>
       <c r="M442" t="s">
         <v>467</v>
       </c>
       <c r="N442" t="s">
-        <v>1387</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="443" spans="1:14">
@@ -14048,7 +14088,7 @@
         <v>156</v>
       </c>
       <c r="K443" t="s">
-        <v>1295</v>
+        <v>1299</v>
       </c>
       <c r="L443" t="s">
         <v>66</v>
@@ -14080,13 +14120,13 @@
         <v>173</v>
       </c>
       <c r="L444" t="s">
-        <v>1359</v>
+        <v>1363</v>
       </c>
       <c r="M444" t="s">
         <v>469</v>
       </c>
       <c r="N444" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="445" spans="1:14">
@@ -14109,13 +14149,13 @@
         <v>173</v>
       </c>
       <c r="L445" t="s">
-        <v>1298</v>
+        <v>1302</v>
       </c>
       <c r="M445" t="s">
         <v>470</v>
       </c>
       <c r="N445" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="446" spans="1:14">
@@ -14138,7 +14178,7 @@
         <v>169</v>
       </c>
       <c r="L446" t="s">
-        <v>1298</v>
+        <v>1302</v>
       </c>
       <c r="M446" t="s">
         <v>471</v>
@@ -14167,7 +14207,7 @@
         <v>175</v>
       </c>
       <c r="L447" t="s">
-        <v>1360</v>
+        <v>1364</v>
       </c>
       <c r="M447" t="s">
         <v>472</v>
@@ -14196,7 +14236,7 @@
         <v>154</v>
       </c>
       <c r="L448" t="s">
-        <v>1333</v>
+        <v>1337</v>
       </c>
       <c r="M448" t="s">
         <v>473</v>
@@ -14231,7 +14271,7 @@
         <v>474</v>
       </c>
       <c r="N449" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="450" spans="1:14">
@@ -14254,13 +14294,13 @@
         <v>175</v>
       </c>
       <c r="L450" t="s">
-        <v>1360</v>
+        <v>1364</v>
       </c>
       <c r="M450" t="s">
         <v>475</v>
       </c>
       <c r="N450" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="451" spans="1:14">
@@ -14283,13 +14323,13 @@
         <v>175</v>
       </c>
       <c r="L451" t="s">
-        <v>1361</v>
+        <v>1365</v>
       </c>
       <c r="M451" t="s">
         <v>476</v>
       </c>
       <c r="N451" t="s">
-        <v>1391</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="452" spans="1:14">
@@ -14312,7 +14352,7 @@
         <v>171</v>
       </c>
       <c r="L452" t="s">
-        <v>1362</v>
+        <v>1366</v>
       </c>
       <c r="M452" t="s">
         <v>477</v>
@@ -14341,13 +14381,13 @@
         <v>171</v>
       </c>
       <c r="L453" t="s">
-        <v>1358</v>
+        <v>1362</v>
       </c>
       <c r="M453" t="s">
         <v>478</v>
       </c>
       <c r="N453" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="454" spans="1:14">
@@ -14405,7 +14445,7 @@
         <v>480</v>
       </c>
       <c r="N455" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="456" spans="1:14">
@@ -14428,13 +14468,13 @@
         <v>173</v>
       </c>
       <c r="L456" t="s">
-        <v>1363</v>
+        <v>1367</v>
       </c>
       <c r="M456" t="s">
         <v>481</v>
       </c>
       <c r="N456" t="s">
-        <v>1403</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="457" spans="1:14">
@@ -14454,10 +14494,10 @@
         <v>156</v>
       </c>
       <c r="K457" t="s">
-        <v>1295</v>
+        <v>1299</v>
       </c>
       <c r="L457" t="s">
-        <v>1333</v>
+        <v>1337</v>
       </c>
       <c r="M457" t="s">
         <v>482</v>
@@ -14486,13 +14526,13 @@
         <v>173</v>
       </c>
       <c r="L458" t="s">
-        <v>1298</v>
+        <v>1302</v>
       </c>
       <c r="M458" t="s">
         <v>483</v>
       </c>
       <c r="N458" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="459" spans="1:14">
@@ -14521,7 +14561,7 @@
         <v>484</v>
       </c>
       <c r="N459" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="460" spans="1:14">
@@ -14544,7 +14584,7 @@
         <v>175</v>
       </c>
       <c r="L460" t="s">
-        <v>1360</v>
+        <v>1364</v>
       </c>
       <c r="M460" t="s">
         <v>485</v>
@@ -14573,13 +14613,13 @@
         <v>175</v>
       </c>
       <c r="L461" t="s">
-        <v>1361</v>
+        <v>1365</v>
       </c>
       <c r="M461" t="s">
         <v>486</v>
       </c>
       <c r="N461" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="462" spans="1:14">
@@ -14602,13 +14642,13 @@
         <v>165</v>
       </c>
       <c r="L462" t="s">
-        <v>1316</v>
+        <v>1320</v>
       </c>
       <c r="M462" t="s">
         <v>487</v>
       </c>
       <c r="N462" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="463" spans="1:14">
@@ -14637,7 +14677,7 @@
         <v>488</v>
       </c>
       <c r="N463" t="s">
-        <v>1403</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="464" spans="1:14">
@@ -14660,13 +14700,13 @@
         <v>173</v>
       </c>
       <c r="L464" t="s">
-        <v>1364</v>
+        <v>1368</v>
       </c>
       <c r="M464" t="s">
         <v>489</v>
       </c>
       <c r="N464" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="465" spans="1:14">
@@ -14689,7 +14729,7 @@
         <v>164</v>
       </c>
       <c r="L465" t="s">
-        <v>1302</v>
+        <v>1306</v>
       </c>
       <c r="M465" t="s">
         <v>490</v>
@@ -14718,13 +14758,13 @@
         <v>164</v>
       </c>
       <c r="L466" t="s">
-        <v>1309</v>
+        <v>1313</v>
       </c>
       <c r="M466" t="s">
         <v>491</v>
       </c>
       <c r="N466" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="467" spans="1:14">
@@ -14753,7 +14793,7 @@
         <v>492</v>
       </c>
       <c r="N467" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="468" spans="1:14">
@@ -14776,13 +14816,13 @@
         <v>164</v>
       </c>
       <c r="L468" t="s">
-        <v>1321</v>
+        <v>1325</v>
       </c>
       <c r="M468" t="s">
         <v>493</v>
       </c>
       <c r="N468" t="s">
-        <v>1384</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="469" spans="1:14">
@@ -14840,7 +14880,7 @@
         <v>495</v>
       </c>
       <c r="N470" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="471" spans="1:14">
@@ -14869,7 +14909,7 @@
         <v>496</v>
       </c>
       <c r="N471" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="472" spans="1:14">
@@ -14886,10 +14926,10 @@
         <v>1095</v>
       </c>
       <c r="G472" s="1" t="s">
-        <v>1268</v>
+        <v>1271</v>
       </c>
       <c r="H472" t="s">
-        <v>1277</v>
+        <v>1281</v>
       </c>
       <c r="J472" t="s">
         <v>155</v>
@@ -14898,13 +14938,13 @@
         <v>165</v>
       </c>
       <c r="L472" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M472" t="s">
         <v>497</v>
       </c>
       <c r="N472" t="s">
-        <v>1391</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="473" spans="1:14">
@@ -14927,7 +14967,7 @@
         <v>165</v>
       </c>
       <c r="L473" t="s">
-        <v>1302</v>
+        <v>1306</v>
       </c>
       <c r="M473" t="s">
         <v>498</v>
@@ -14985,13 +15025,13 @@
         <v>170</v>
       </c>
       <c r="L475" t="s">
-        <v>1365</v>
+        <v>1369</v>
       </c>
       <c r="M475" t="s">
         <v>500</v>
       </c>
       <c r="N475" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="476" spans="1:14">
@@ -15014,13 +15054,13 @@
         <v>173</v>
       </c>
       <c r="L476" t="s">
-        <v>1356</v>
+        <v>1360</v>
       </c>
       <c r="M476" t="s">
         <v>501</v>
       </c>
       <c r="N476" t="s">
-        <v>1387</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="477" spans="1:14">
@@ -15036,6 +15076,9 @@
       <c r="D477" t="s">
         <v>1100</v>
       </c>
+      <c r="E477" t="s">
+        <v>1265</v>
+      </c>
       <c r="J477" t="s">
         <v>156</v>
       </c>
@@ -15043,13 +15086,13 @@
         <v>173</v>
       </c>
       <c r="L477" t="s">
-        <v>1366</v>
+        <v>1370</v>
       </c>
       <c r="M477" t="s">
         <v>502</v>
       </c>
       <c r="N477" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="478" spans="1:14">
@@ -15072,13 +15115,13 @@
         <v>170</v>
       </c>
       <c r="L478" t="s">
-        <v>1309</v>
+        <v>1313</v>
       </c>
       <c r="M478" t="s">
         <v>503</v>
       </c>
       <c r="N478" t="s">
-        <v>1409</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="479" spans="1:14">
@@ -15101,13 +15144,13 @@
         <v>173</v>
       </c>
       <c r="L479" t="s">
-        <v>1298</v>
+        <v>1302</v>
       </c>
       <c r="M479" t="s">
         <v>504</v>
       </c>
       <c r="N479" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="480" spans="1:14">
@@ -15130,7 +15173,7 @@
         <v>173</v>
       </c>
       <c r="L480" t="s">
-        <v>1367</v>
+        <v>1371</v>
       </c>
       <c r="M480" t="s">
         <v>505</v>
@@ -15159,7 +15202,7 @@
         <v>173</v>
       </c>
       <c r="L481" t="s">
-        <v>1366</v>
+        <v>1370</v>
       </c>
       <c r="M481" t="s">
         <v>506</v>
@@ -15188,13 +15231,13 @@
         <v>173</v>
       </c>
       <c r="L482" t="s">
-        <v>1348</v>
+        <v>1352</v>
       </c>
       <c r="M482" t="s">
         <v>507</v>
       </c>
       <c r="N482" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="483" spans="1:14">
@@ -15217,13 +15260,13 @@
         <v>173</v>
       </c>
       <c r="L483" t="s">
-        <v>1368</v>
+        <v>1372</v>
       </c>
       <c r="M483" t="s">
         <v>508</v>
       </c>
       <c r="N483" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="484" spans="1:14">
@@ -15252,7 +15295,7 @@
         <v>509</v>
       </c>
       <c r="N484" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="485" spans="1:14">
@@ -15275,7 +15318,7 @@
         <v>173</v>
       </c>
       <c r="L485" t="s">
-        <v>1336</v>
+        <v>1340</v>
       </c>
       <c r="M485" t="s">
         <v>510</v>
@@ -15304,13 +15347,13 @@
         <v>67</v>
       </c>
       <c r="L486" t="s">
-        <v>1298</v>
+        <v>1302</v>
       </c>
       <c r="M486" t="s">
         <v>511</v>
       </c>
       <c r="N486" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="487" spans="1:14">
@@ -15333,13 +15376,13 @@
         <v>67</v>
       </c>
       <c r="L487" t="s">
-        <v>1369</v>
+        <v>1373</v>
       </c>
       <c r="M487" t="s">
         <v>512</v>
       </c>
       <c r="N487" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="488" spans="1:14">
@@ -15362,13 +15405,13 @@
         <v>67</v>
       </c>
       <c r="L488" t="s">
-        <v>1309</v>
+        <v>1313</v>
       </c>
       <c r="M488" t="s">
         <v>513</v>
       </c>
       <c r="N488" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="489" spans="1:14">
@@ -15391,13 +15434,13 @@
         <v>172</v>
       </c>
       <c r="L489" t="s">
-        <v>1370</v>
+        <v>1374</v>
       </c>
       <c r="M489" t="s">
         <v>514</v>
       </c>
       <c r="N489" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="490" spans="1:14">
@@ -15420,13 +15463,13 @@
         <v>172</v>
       </c>
       <c r="L490" t="s">
-        <v>1333</v>
+        <v>1337</v>
       </c>
       <c r="M490" t="s">
         <v>515</v>
       </c>
       <c r="N490" t="s">
-        <v>1391</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="491" spans="1:14">
@@ -15449,13 +15492,13 @@
         <v>175</v>
       </c>
       <c r="L491" t="s">
-        <v>1371</v>
+        <v>1375</v>
       </c>
       <c r="M491" t="s">
         <v>516</v>
       </c>
       <c r="N491" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="492" spans="1:14">
@@ -15472,7 +15515,7 @@
         <v>1115</v>
       </c>
       <c r="H492" t="s">
-        <v>1278</v>
+        <v>1282</v>
       </c>
       <c r="J492" t="s">
         <v>155</v>
@@ -15487,7 +15530,7 @@
         <v>517</v>
       </c>
       <c r="N492" t="s">
-        <v>1392</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="493" spans="1:14">
@@ -15507,13 +15550,13 @@
         <v>167</v>
       </c>
       <c r="L493" t="s">
-        <v>1318</v>
+        <v>1322</v>
       </c>
       <c r="M493" t="s">
         <v>518</v>
       </c>
       <c r="N493" t="s">
-        <v>1406</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="494" spans="1:14">
@@ -15530,7 +15573,7 @@
         <v>1116</v>
       </c>
       <c r="H494" t="s">
-        <v>1279</v>
+        <v>1283</v>
       </c>
       <c r="J494" t="s">
         <v>155</v>
@@ -15568,7 +15611,7 @@
         <v>168</v>
       </c>
       <c r="L495" t="s">
-        <v>1372</v>
+        <v>1376</v>
       </c>
       <c r="M495" t="s">
         <v>520</v>
@@ -15597,13 +15640,13 @@
         <v>168</v>
       </c>
       <c r="L496" t="s">
-        <v>1350</v>
+        <v>1354</v>
       </c>
       <c r="M496" t="s">
         <v>521</v>
       </c>
       <c r="N496" t="s">
-        <v>1387</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="497" spans="1:14">
@@ -15623,16 +15666,16 @@
         <v>156</v>
       </c>
       <c r="K497" t="s">
-        <v>1296</v>
+        <v>1300</v>
       </c>
       <c r="L497" t="s">
-        <v>1325</v>
+        <v>1329</v>
       </c>
       <c r="M497" t="s">
         <v>522</v>
       </c>
       <c r="N497" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="498" spans="1:14">
@@ -15655,13 +15698,13 @@
         <v>168</v>
       </c>
       <c r="L498" t="s">
-        <v>1373</v>
+        <v>1377</v>
       </c>
       <c r="M498" t="s">
         <v>523</v>
       </c>
       <c r="N498" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="499" spans="1:14">
@@ -15684,13 +15727,13 @@
         <v>169</v>
       </c>
       <c r="L499" t="s">
-        <v>1308</v>
+        <v>1312</v>
       </c>
       <c r="M499" t="s">
         <v>524</v>
       </c>
       <c r="N499" t="s">
-        <v>1410</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="500" spans="1:14">
@@ -15719,7 +15762,7 @@
         <v>525</v>
       </c>
       <c r="N500" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="501" spans="1:14">
@@ -15742,13 +15785,13 @@
         <v>170</v>
       </c>
       <c r="L501" t="s">
-        <v>1315</v>
+        <v>1319</v>
       </c>
       <c r="M501" t="s">
         <v>526</v>
       </c>
       <c r="N501" t="s">
-        <v>1395</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="502" spans="1:14">
@@ -15771,13 +15814,13 @@
         <v>167</v>
       </c>
       <c r="L502" t="s">
-        <v>1300</v>
+        <v>1304</v>
       </c>
       <c r="M502" t="s">
         <v>527</v>
       </c>
       <c r="N502" t="s">
-        <v>1396</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="503" spans="1:14">
@@ -15800,7 +15843,7 @@
         <v>172</v>
       </c>
       <c r="L503" t="s">
-        <v>1348</v>
+        <v>1352</v>
       </c>
       <c r="M503" t="s">
         <v>528</v>
@@ -15829,7 +15872,7 @@
         <v>175</v>
       </c>
       <c r="L504" t="s">
-        <v>1317</v>
+        <v>1321</v>
       </c>
       <c r="M504" t="s">
         <v>529</v>
@@ -15893,7 +15936,7 @@
         <v>531</v>
       </c>
       <c r="N506" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="507" spans="1:14">
@@ -15916,13 +15959,13 @@
         <v>164</v>
       </c>
       <c r="L507" t="s">
-        <v>1334</v>
+        <v>1338</v>
       </c>
       <c r="M507" t="s">
         <v>532</v>
       </c>
       <c r="N507" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="508" spans="1:14">
@@ -15945,13 +15988,13 @@
         <v>166</v>
       </c>
       <c r="L508" t="s">
-        <v>1374</v>
+        <v>1378</v>
       </c>
       <c r="M508" t="s">
         <v>533</v>
       </c>
       <c r="N508" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="509" spans="1:14">
@@ -15974,7 +16017,7 @@
         <v>165</v>
       </c>
       <c r="L509" t="s">
-        <v>1309</v>
+        <v>1313</v>
       </c>
       <c r="M509" t="s">
         <v>534</v>
@@ -16009,7 +16052,7 @@
         <v>535</v>
       </c>
       <c r="N510" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="511" spans="1:14">
@@ -16038,7 +16081,7 @@
         <v>536</v>
       </c>
       <c r="N511" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="512" spans="1:14">
@@ -16067,7 +16110,7 @@
         <v>537</v>
       </c>
       <c r="N512" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="513" spans="1:14">
@@ -16096,7 +16139,7 @@
         <v>538</v>
       </c>
       <c r="N513" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="514" spans="1:14">
@@ -16148,7 +16191,7 @@
         <v>167</v>
       </c>
       <c r="L515" t="s">
-        <v>1323</v>
+        <v>1327</v>
       </c>
       <c r="M515" t="s">
         <v>540</v>
@@ -16206,7 +16249,7 @@
         <v>171</v>
       </c>
       <c r="L517" t="s">
-        <v>1375</v>
+        <v>1379</v>
       </c>
       <c r="M517" t="s">
         <v>542</v>
@@ -16241,7 +16284,7 @@
         <v>543</v>
       </c>
       <c r="N518" t="s">
-        <v>1388</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="519" spans="1:14">
@@ -16270,7 +16313,7 @@
         <v>544</v>
       </c>
       <c r="N519" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="520" spans="1:14">
@@ -16293,13 +16336,13 @@
         <v>170</v>
       </c>
       <c r="L520" t="s">
-        <v>1308</v>
+        <v>1312</v>
       </c>
       <c r="M520" t="s">
         <v>545</v>
       </c>
       <c r="N520" t="s">
-        <v>1393</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="521" spans="1:14">
@@ -16322,13 +16365,13 @@
         <v>170</v>
       </c>
       <c r="L521" t="s">
-        <v>1376</v>
+        <v>1380</v>
       </c>
       <c r="M521" t="s">
         <v>546</v>
       </c>
       <c r="N521" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="522" spans="1:14">
@@ -16351,7 +16394,7 @@
         <v>167</v>
       </c>
       <c r="L522" t="s">
-        <v>1377</v>
+        <v>1381</v>
       </c>
       <c r="M522" t="s">
         <v>547</v>
@@ -16386,7 +16429,7 @@
         <v>548</v>
       </c>
       <c r="N523" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="524" spans="1:14">
@@ -16409,13 +16452,13 @@
         <v>166</v>
       </c>
       <c r="L524" t="s">
-        <v>1378</v>
+        <v>1382</v>
       </c>
       <c r="M524" t="s">
         <v>549</v>
       </c>
       <c r="N524" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="525" spans="1:14">
@@ -16438,13 +16481,13 @@
         <v>173</v>
       </c>
       <c r="L525" t="s">
-        <v>1379</v>
+        <v>1383</v>
       </c>
       <c r="M525" t="s">
         <v>550</v>
       </c>
       <c r="N525" t="s">
-        <v>1383</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="526" spans="1:14">
@@ -16496,7 +16539,7 @@
         <v>167</v>
       </c>
       <c r="L527" t="s">
-        <v>1302</v>
+        <v>1306</v>
       </c>
       <c r="M527" t="s">
         <v>552</v>
@@ -16525,13 +16568,13 @@
         <v>167</v>
       </c>
       <c r="L528" t="s">
-        <v>1318</v>
+        <v>1322</v>
       </c>
       <c r="M528" t="s">
         <v>553</v>
       </c>
       <c r="N528" t="s">
-        <v>1392</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="529" spans="1:14">
@@ -16554,13 +16597,13 @@
         <v>172</v>
       </c>
       <c r="L529" t="s">
-        <v>1299</v>
+        <v>1303</v>
       </c>
       <c r="M529" t="s">
         <v>554</v>
       </c>
       <c r="N529" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="530" spans="1:14">
@@ -16583,13 +16626,13 @@
         <v>170</v>
       </c>
       <c r="L530" t="s">
-        <v>1335</v>
+        <v>1339</v>
       </c>
       <c r="M530" t="s">
         <v>555</v>
       </c>
       <c r="N530" t="s">
-        <v>1384</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="531" spans="1:14">
@@ -16612,13 +16655,13 @@
         <v>170</v>
       </c>
       <c r="L531" t="s">
-        <v>1380</v>
+        <v>1384</v>
       </c>
       <c r="M531" t="s">
         <v>556</v>
       </c>
       <c r="N531" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="532" spans="1:14">
@@ -16670,13 +16713,13 @@
         <v>166</v>
       </c>
       <c r="L533" t="s">
-        <v>1381</v>
+        <v>1385</v>
       </c>
       <c r="M533" t="s">
         <v>558</v>
       </c>
       <c r="N533" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="534" spans="1:14">
@@ -16705,7 +16748,7 @@
         <v>559</v>
       </c>
       <c r="N534" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="535" spans="1:14">
@@ -16728,13 +16771,13 @@
         <v>67</v>
       </c>
       <c r="L535" t="s">
-        <v>1382</v>
+        <v>1386</v>
       </c>
       <c r="M535" t="s">
         <v>560</v>
       </c>
       <c r="N535" t="s">
-        <v>1386</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="536" spans="1:14">
@@ -16877,7 +16920,7 @@
         <v>1167</v>
       </c>
       <c r="H545" t="s">
-        <v>1280</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="546" spans="1:8">

</xml_diff>